<commit_message>
Update default config to Mikrotik-TP3.rsc, update excels, and commit artifacts
</commit_message>
<xml_diff>
--- a/A-Draft - Mikrotik Deployment.xlsx
+++ b/A-Draft - Mikrotik Deployment.xlsx
@@ -7527,7 +7527,7 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>add action=accept chain=forward comment= "[02-A] ALLOW ICMP (PING) FOR POC VERIFICATION" protocol=icmp</t>
+          <t>add action=accept chain=forward comment= "[03] ALLOW ICMP (PING) FOR VERIFICATION" protocol=icmp</t>
         </is>
       </c>
     </row>
@@ -7561,14 +7561,14 @@
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>add action=accept chain=forward comment= "[03] ALLOW PUBLIC WEB TRAFFIC TO WAF" dst-address-list=waf-frontend  dst-port=80,443 protocol=tcp</t>
+          <t>add action=accept chain=forward comment= "[03-A] ALLOW PUBLIC WEB TRAFFIC TO WAF" dst-address-list=waf-frontend  dst-port=80,443 protocol=tcp</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>02-B</t>
+          <t>03-B</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -7598,12 +7598,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>[02-B] ALLOW WAF TO BACKEND APACHE</t>
+          <t>[03-B] ALLOW WAF TO BACKEND APACHE</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>add action=accept chain=forward comment="[02-B] ALLOW WAF TO BACKEND APACHE"  dst-address=10.27.101.165 dst-port=8881 protocol=tcp src-address= 10.27.101.41</t>
+          <t>add action=accept chain=forward comment="[03-B] ALLOW WAF TO BACKEND APACHE"  dst-address=10.27.101.165 dst-port=8881 protocol=tcp src-address= 10.27.101.41</t>
         </is>
       </c>
     </row>

</xml_diff>